<commit_message>
Gestion de facture opérationnelle
</commit_message>
<xml_diff>
--- a/ExcelFiles/Produits.xlsx
+++ b/ExcelFiles/Produits.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -610,6 +610,21 @@
         <v>12</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P0078</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>bonbon</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>